<commit_message>
Weekly data update from SharePoint
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -54187,15 +54187,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CFB2F24-829F-4D5B-9EB0-E261189A0819}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A1E5B5D-04A9-44F8-BDC1-A1CF40A7D271}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{425A0947-A89D-4F60-B701-6B6C9110ED81}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A3D0802-6E62-44EF-9689-88741942C570}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{614FB914-D9BD-419A-BD8C-9B997AC88862}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5E3D562-33C5-4C2A-972E-2D7AD8817191}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>